<commit_message>
fixed - This card
</commit_message>
<xml_diff>
--- a/Book1-Vocabulary.xlsx
+++ b/Book1-Vocabulary.xlsx
@@ -81,7 +81,7 @@
     <t xml:space="preserve">هَذَا</t>
   </si>
   <si>
-    <t xml:space="preserve">this (m., near)</t>
+    <t xml:space="preserve">this (m.)</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -894,7 +894,7 @@
     <t xml:space="preserve">هَذِهِ</t>
   </si>
   <si>
-    <t xml:space="preserve">this (f., near)</t>
+    <t xml:space="preserve">this (f.)</t>
   </si>
   <si>
     <t xml:space="preserve">تِلْكَ</t>
@@ -1308,7 +1308,7 @@
     <t xml:space="preserve">More هَذَا sentences. Nouns ending in ـٌ are indefinite ("a book"). Every Arabic noun has a gender — masculine or feminine.</t>
   </si>
   <si>
-    <t xml:space="preserve">More هَذَا/ذَلِكَ with animals. All these nouns are masculine. وَ means "and" — it attaches directly to the next word: هَذَا فِيلٌ وَذَلِكَ جَمَلٌ. Note: عَنْكَبُوتٌ (spider) takes either gender — we treat it as masculine here, though the Quran uses a feminine verb with it in Sūrat al-ʿAnkabūt.</t>
+    <t xml:space="preserve">More هَذَا/ذَلِكَ with animals. All these nouns are masculine. وَ means "and" — it attaches directly to the next word: هَذَا فِيلٌ وَذَلِكَ جَمَلٌ. Note: عَنْكَبُوتٌ (spider) can be treated as masculine or feminine; we use هَذَا with it here.</t>
   </si>
   <si>
     <t xml:space="preserve">مَنْ هَذَا؟ = Who is this? Used for people: مَنْ هَذَا؟ هَذَا إِمَامٌ. مَا هَذَا؟ هَذَا قَمِيصٌ.</t>

</xml_diff>